<commit_message>
Rebrand header, drop footer line, handle in-progress seasons
- Header and homepage title become 蒂亚鸽のFantasy Portfolio; tagline is now
  蒂亚鸽鸽鸽/TheViolin/TheViolin233 的范特西档案
- Remove the "Updated monthly from a spreadsheet" footer line
- Season rows with no points, rank or percentile yet render an "In progress"
  badge instead of a grid of em dashes, matching how ongoing mini-leagues
  already read. Covers the new fpl and f1 2026-27 rows.
- Align the league card's accent dot to the first line of the title, since
  the new Chinese-parenthetical names wrap to two lines
- Stop long mini-league hosts ("The Forbidden Endzone") from pushing their
  status badge onto a second line

Picks up the new NBA and NFL leagues and the NFL draft leagues from the
workbook; both new categories render without any code change.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/fantasy-portfolio.xlsx
+++ b/data/fantasy-portfolio.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13061EB-5182-4E80-848C-045DDC50FF02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4ECCEEA-0F09-40E9-9C5B-9E91D9C0E353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="73">
   <si>
     <t>slug</t>
   </si>
@@ -40,12 +40,6 @@
     <t>fpl</t>
   </si>
   <si>
-    <t>Fantasy Premier League</t>
-  </si>
-  <si>
-    <t>Soccer Official</t>
-  </si>
-  <si>
     <t>Soccer</t>
   </si>
   <si>
@@ -58,151 +52,226 @@
     <t>f1</t>
   </si>
   <si>
+    <t>Motorsport</t>
+  </si>
+  <si>
+    <t>#ff1e00</t>
+  </si>
+  <si>
+    <t>wc</t>
+  </si>
+  <si>
+    <t>#008057</t>
+  </si>
+  <si>
+    <t>uefa</t>
+  </si>
+  <si>
+    <t>#4dffff</t>
+  </si>
+  <si>
+    <t>league</t>
+  </si>
+  <si>
+    <t>season</t>
+  </si>
+  <si>
+    <t>team_name</t>
+  </si>
+  <si>
+    <t>points</t>
+  </si>
+  <si>
+    <t>overall_rank</t>
+  </si>
+  <si>
+    <t>total_players</t>
+  </si>
+  <si>
+    <t>pct_finish</t>
+  </si>
+  <si>
+    <t>mini_league</t>
+  </si>
+  <si>
+    <t>mini_league_rank</t>
+  </si>
+  <si>
+    <t>mini_league_size</t>
+  </si>
+  <si>
+    <t>result</t>
+  </si>
+  <si>
+    <t>highlight</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>2025-26</t>
+  </si>
+  <si>
+    <t>6%</t>
+  </si>
+  <si>
+    <t>2024-25</t>
+  </si>
+  <si>
+    <t>56%</t>
+  </si>
+  <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>fpl</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025-26</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>蒂亚鸽鸽鸽</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>企鹅联赛</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>2026-27</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>mini_league_host</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>mini_league_format</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>蒂亚鸽鸽鸽（联赛版）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>wc</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>蒂亚鸽鸽鸽（北极奥地利）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>mini_league_result</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>小组未出线</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>很早淘汰</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>uefa</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>队长对战</t>
+  </si>
+  <si>
+    <t>队长对战</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>No Big 6</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>f1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>nba</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>nfl</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>NBA Fantasy</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Basketball</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>NFL Fantasy</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Football</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fantasy Premier League (英超范特西)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>F1 Fantasy</t>
-  </si>
-  <si>
-    <t>F1 Official</t>
-  </si>
-  <si>
-    <t>Motorsport</t>
-  </si>
-  <si>
-    <t>#ff1e00</t>
-  </si>
-  <si>
-    <t>wc</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>World Cup</t>
-  </si>
-  <si>
-    <t>#008057</t>
-  </si>
-  <si>
-    <t>uefa</t>
-  </si>
-  <si>
-    <t>Champions League Fantasy</t>
-  </si>
-  <si>
-    <t>#4dffff</t>
-  </si>
-  <si>
-    <t>league</t>
-  </si>
-  <si>
-    <t>season</t>
-  </si>
-  <si>
-    <t>team_name</t>
-  </si>
-  <si>
-    <t>points</t>
-  </si>
-  <si>
-    <t>overall_rank</t>
-  </si>
-  <si>
-    <t>total_players</t>
-  </si>
-  <si>
-    <t>pct_finish</t>
-  </si>
-  <si>
-    <t>mini_league</t>
-  </si>
-  <si>
-    <t>mini_league_rank</t>
-  </si>
-  <si>
-    <t>mini_league_size</t>
-  </si>
-  <si>
-    <t>result</t>
-  </si>
-  <si>
-    <t>highlight</t>
-  </si>
-  <si>
-    <t>notes</t>
-  </si>
-  <si>
-    <t>2025-26</t>
-  </si>
-  <si>
-    <t>6%</t>
-  </si>
-  <si>
-    <t>2024-25</t>
-  </si>
-  <si>
-    <t>56%</t>
-  </si>
-  <si>
-    <t>2026</t>
-  </si>
-  <si>
-    <t>fpl</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>2025-26</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>蒂亚鸽鸽鸽</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>企鹅联赛</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>2026-27</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>mini_league_host</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>mini_league_format</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>队长vs</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>无Big6</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>蒂亚鸽鸽鸽（联赛版）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>wc</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>世界杯赛制</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>蒂亚鸽鸽鸽（北极奥地利）</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>mini_league_result</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>小组未出线</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>很早淘汰</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Champions League Fantasy (欧冠范特西)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>九麦联赛</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>#1D428A</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>#835737</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Yahoo Redraft</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>The Forbidden Endzone</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dynasty</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>足球</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>赛车</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>篮球</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>橄榄球</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -603,11 +672,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.1"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="2" max="2" width="39" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="11" customWidth="1"/>
@@ -639,79 +708,113 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
       <c r="D4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
         <v>9</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
       <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
         <v>9</v>
       </c>
-      <c r="E5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -723,7 +826,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="14.1"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -741,43 +844,43 @@
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="J1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="K1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="L1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="M1" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -785,7 +888,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D2" s="2">
         <v>2216</v>
@@ -794,7 +897,7 @@
         <v>737806</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -802,7 +905,7 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D3" s="2">
         <v>1917</v>
@@ -811,15 +914,15 @@
         <v>6349372</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D4" s="2">
         <v>1257</v>
@@ -828,15 +931,15 @@
         <v>44953</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D5" s="2">
         <v>645</v>
@@ -845,7 +948,23 @@
         <v>228129</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -857,7 +976,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B23D03EC-9F84-4107-AC36-AB27839C1362}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.1"/>
   <cols>
     <col min="3" max="4" width="18.15625" bestFit="1" customWidth="1"/>
@@ -867,96 +986,138 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E3" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E4" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="B5">
         <v>2026</v>
       </c>
       <c r="C5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" t="s">
         <v>44</v>
       </c>
-      <c r="D5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E5" t="s">
-        <v>53</v>
-      </c>
       <c r="F5" t="s">
-        <v>55</v>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>